<commit_message>
Dodaje plik interfejsu: -AdminInterface
Dodaje zmienną i funkcję do GlobalVariables:
-isAdmin
- funkcja checkAdmin

Dodałem formularz usuwania i dodawania książek

Zmieniłem styl graficzny
Poprawiłem kod w moich plikach
podpiołem funkcję kupowania książek

zmieniłem bazę danych (book.xlsx):
-zamieniłem tekst na wiersze i kolumny

Dodałem zdjęcie jako bazowa okładka książki
</commit_message>
<xml_diff>
--- a/DATABASE/book.xlsx
+++ b/DATABASE/book.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\FR1PEPF00001169\EXCELCNV\65d635ba-622d-4214-8c40-bd9c21ababd3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{798B7F13-109E-431F-8CD0-08C87080E20E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0E6AE8F-47A1-4C12-B811-77BDAF81D603}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA60D7CB-0065-43BF-A6BC-971827DF2C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{6502C133-150D-4F54-88C8-31CE5A5F8E12}"/>
   </bookViews>
@@ -36,18 +36,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>ID,AUTHOR,TITLE,NO_EBOOK_AVAILABLE,CREATED,UPDATED</t>
-  </si>
-  <si>
-    <t>101,David Kahn,The Codebreakers,1200,2018-03-15,2018-03-17</t>
-  </si>
-  <si>
-    <t>102,Donald Knuth,The Art of Computer Programming,3168,2018-03-15,2018-03-15</t>
-  </si>
-  <si>
-    <t>103,Matt Weisfeld,The Object-Oriented Thought Process,336,2018-03-15,2018-03-18</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>AUTHOR</t>
+  </si>
+  <si>
+    <t>TITLE</t>
+  </si>
+  <si>
+    <t>NO_EBOOK_AVAILABLE</t>
+  </si>
+  <si>
+    <t>CREATED</t>
+  </si>
+  <si>
+    <t>UPDATED</t>
+  </si>
+  <si>
+    <t>David Kahn</t>
+  </si>
+  <si>
+    <t>The Codebreakers</t>
+  </si>
+  <si>
+    <t>Donald Knuth</t>
+  </si>
+  <si>
+    <t>The Art of Computer Programming</t>
+  </si>
+  <si>
+    <t>Matt Weisfeld</t>
+  </si>
+  <si>
+    <t>The Object-Oriented Thought Process</t>
+  </si>
+  <si>
+    <t>Andrzej Sapkowski</t>
+  </si>
+  <si>
+    <t>Wiedźmin: Ostatnie życzenie</t>
   </si>
 </sst>
 </file>
@@ -549,52 +579,53 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% — akcent 6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% — akcent 6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% — akcent 6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Akcent 1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Akcent 2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Akcent 3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Akcent 4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Akcent 5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Akcent 6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Dane wejściowe" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Dane wyjściowe" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Dobry" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Komórka połączona" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Komórka zaznaczona" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Nagłówek 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Nagłówek 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Nagłówek 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Nagłówek 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Neutralny" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Obliczenia" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Suma" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Tekst objaśnienia" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Tekst ostrzeżenia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Tytuł" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Uwaga" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Zły" xfId="7" builtinId="27" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -906,27 +937,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60826CDF-661A-4289-9A79-FA33799C86AD}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="39.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>1</v>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>1200</v>
+      </c>
+      <c r="E2" s="1">
+        <v>43174</v>
+      </c>
+      <c r="F2" s="1">
+        <v>43176</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>2</v>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>3168</v>
+      </c>
+      <c r="E3" s="1">
+        <v>43174</v>
+      </c>
+      <c r="F3" s="1">
+        <v>43174</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>3</v>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>336</v>
+      </c>
+      <c r="E4" s="1">
+        <v>43174</v>
+      </c>
+      <c r="F4" s="1">
+        <v>43177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>1500</v>
+      </c>
+      <c r="E5" s="1">
+        <v>43174</v>
+      </c>
+      <c r="F5" s="1">
+        <v>43174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>